<commit_message>
Update MLB hitter fantasy scores 2026-07-24 (2026-07-23 10:03 PM)
</commit_message>
<xml_diff>
--- a/PRIZEPICKS_HITTER_AI_V5_TOP30_2026_07_24.xlsx
+++ b/PRIZEPICKS_HITTER_AI_V5_TOP30_2026_07_24.xlsx
@@ -7218,10 +7218,10 @@
         <v>10.75</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>8.81</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>8.81</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>7.08</v>
@@ -7296,10 +7296,10 @@
         <v>54.1</v>
       </c>
       <c r="AI8" s="7" t="n">
-        <v>46.5</v>
+        <v>46.4</v>
       </c>
       <c r="AJ8" s="7" t="n">
-        <v>45</v>
+        <v>44.9</v>
       </c>
       <c r="AK8" s="7" t="n">
         <v>40.7</v>
@@ -7311,10 +7311,10 @@
         <v>36.5</v>
       </c>
       <c r="AN8" s="8" t="n">
-        <v>32.7</v>
+        <v>32.6</v>
       </c>
       <c r="AO8" s="8" t="n">
-        <v>32.7</v>
+        <v>32.6</v>
       </c>
       <c r="AP8" s="8" t="n">
         <v>30.4</v>
@@ -7323,10 +7323,10 @@
         <v>30.4</v>
       </c>
       <c r="AR8" s="8" t="n">
-        <v>27.9</v>
+        <v>27.8</v>
       </c>
       <c r="AS8" s="8" t="n">
-        <v>27.9</v>
+        <v>27.8</v>
       </c>
       <c r="AT8" s="8" t="n">
         <v>26.3</v>
@@ -7341,13 +7341,13 @@
         <v>21.6</v>
       </c>
       <c r="AX8" s="8" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
       <c r="AY8" s="8" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
       <c r="AZ8" s="3" t="n">
-        <v>239.05</v>
+        <v>238.89</v>
       </c>
       <c r="BA8" s="4" t="inlineStr">
         <is>
@@ -7371,7 +7371,7 @@
         <v>58.4</v>
       </c>
       <c r="BF8" s="3" t="n">
-        <v>2.81</v>
+        <v>2.8</v>
       </c>
       <c r="BG8" s="3" t="n">
         <v>16.8</v>
@@ -7837,13 +7837,13 @@
         <v>7.7</v>
       </c>
       <c r="GT8" s="3" t="n">
-        <v>3.25</v>
+        <v>3.24</v>
       </c>
       <c r="GU8" s="3" t="n">
         <v>13.78</v>
       </c>
       <c r="GV8" s="3" t="n">
-        <v>19.52</v>
+        <v>19.53</v>
       </c>
       <c r="GW8" s="3" t="n">
         <v>4.49</v>
@@ -7892,10 +7892,10 @@
         <v>51.1</v>
       </c>
       <c r="HK8" s="3" t="n">
-        <v>44</v>
+        <v>43.9</v>
       </c>
       <c r="HL8" s="3" t="n">
-        <v>44</v>
+        <v>43.9</v>
       </c>
       <c r="HM8" s="3" t="n">
         <v>40.7</v>
@@ -7907,10 +7907,10 @@
         <v>36.5</v>
       </c>
       <c r="HP8" s="3" t="n">
-        <v>32.7</v>
+        <v>32.6</v>
       </c>
       <c r="HQ8" s="3" t="n">
-        <v>32.7</v>
+        <v>32.6</v>
       </c>
       <c r="HR8" s="3" t="n">
         <v>30.4</v>
@@ -7919,10 +7919,10 @@
         <v>30.4</v>
       </c>
       <c r="HT8" s="3" t="n">
-        <v>27.9</v>
+        <v>27.8</v>
       </c>
       <c r="HU8" s="3" t="n">
-        <v>27.9</v>
+        <v>27.8</v>
       </c>
       <c r="HV8" s="3" t="n">
         <v>26.3</v>
@@ -7937,10 +7937,10 @@
         <v>21.6</v>
       </c>
       <c r="HZ8" s="3" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
       <c r="IA8" s="3" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
       <c r="IB8" s="3" t="n">
         <v>8</v>
@@ -21686,10 +21686,10 @@
         <v>9.73</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>9.02</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>9.02</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>6.4</v>
@@ -21707,7 +21707,7 @@
         <v>7.34</v>
       </c>
       <c r="R25" s="3" t="n">
-        <v>0.869</v>
+        <v>0.868</v>
       </c>
       <c r="S25" s="3" t="n">
         <v>6.2</v>
@@ -21749,19 +21749,19 @@
         <v>73.09999999999999</v>
       </c>
       <c r="AD25" s="5" t="n">
-        <v>67.5</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="AE25" s="5" t="n">
-        <v>67</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="AF25" s="6" t="n">
-        <v>57.1</v>
+        <v>57.2</v>
       </c>
       <c r="AG25" s="7" t="n">
-        <v>53.2</v>
+        <v>53.3</v>
       </c>
       <c r="AH25" s="7" t="n">
-        <v>52.7</v>
+        <v>52.8</v>
       </c>
       <c r="AI25" s="7" t="n">
         <v>46.1</v>
@@ -21770,25 +21770,25 @@
         <v>44.6</v>
       </c>
       <c r="AK25" s="8" t="n">
-        <v>39.8</v>
+        <v>39.9</v>
       </c>
       <c r="AL25" s="8" t="n">
-        <v>39.8</v>
+        <v>39.9</v>
       </c>
       <c r="AM25" s="8" t="n">
         <v>36.6</v>
       </c>
       <c r="AN25" s="8" t="n">
-        <v>33.5</v>
+        <v>33.6</v>
       </c>
       <c r="AO25" s="8" t="n">
-        <v>33.5</v>
+        <v>33.6</v>
       </c>
       <c r="AP25" s="8" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="AQ25" s="8" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="AR25" s="8" t="n">
         <v>30.2</v>
@@ -21815,7 +21815,7 @@
         <v>19.1</v>
       </c>
       <c r="AZ25" s="3" t="n">
-        <v>221.19</v>
+        <v>221.36</v>
       </c>
       <c r="BA25" s="4" t="inlineStr">
         <is>
@@ -21824,7 +21824,7 @@
       </c>
       <c r="BB25" s="9" t="inlineStr">
         <is>
-          <t>MORE 5.5 | 67.0% | Edge +3.5</t>
+          <t>MORE 5.5 | 67.1% | Edge +3.5</t>
         </is>
       </c>
       <c r="BC25" s="4" t="inlineStr">
@@ -21836,13 +21836,13 @@
         <v>5.5</v>
       </c>
       <c r="BE25" s="3" t="n">
-        <v>67</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="BF25" s="3" t="n">
-        <v>3.52</v>
+        <v>3.53</v>
       </c>
       <c r="BG25" s="3" t="n">
-        <v>34</v>
+        <v>34.2</v>
       </c>
       <c r="BH25" s="4" t="inlineStr">
         <is>
@@ -22311,7 +22311,7 @@
         <v>13.35</v>
       </c>
       <c r="GV25" s="3" t="n">
-        <v>19.43</v>
+        <v>19.42</v>
       </c>
       <c r="GW25" s="3" t="n">
         <v>4.65</v>
@@ -22345,19 +22345,19 @@
         <v>67.09999999999999</v>
       </c>
       <c r="HF25" s="3" t="n">
-        <v>62.5</v>
+        <v>62.6</v>
       </c>
       <c r="HG25" s="3" t="n">
-        <v>62.5</v>
+        <v>62.6</v>
       </c>
       <c r="HH25" s="3" t="n">
-        <v>53.1</v>
+        <v>53.2</v>
       </c>
       <c r="HI25" s="3" t="n">
-        <v>49.7</v>
+        <v>49.8</v>
       </c>
       <c r="HJ25" s="3" t="n">
-        <v>49.7</v>
+        <v>49.8</v>
       </c>
       <c r="HK25" s="3" t="n">
         <v>43.6</v>
@@ -22366,25 +22366,25 @@
         <v>43.6</v>
       </c>
       <c r="HM25" s="3" t="n">
-        <v>39.8</v>
+        <v>39.9</v>
       </c>
       <c r="HN25" s="3" t="n">
-        <v>39.8</v>
+        <v>39.9</v>
       </c>
       <c r="HO25" s="3" t="n">
         <v>36.6</v>
       </c>
       <c r="HP25" s="3" t="n">
-        <v>33.5</v>
+        <v>33.6</v>
       </c>
       <c r="HQ25" s="3" t="n">
-        <v>33.5</v>
+        <v>33.6</v>
       </c>
       <c r="HR25" s="3" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="HS25" s="3" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="HT25" s="3" t="n">
         <v>30.2</v>
@@ -22506,22 +22506,22 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Drake Baldwin</t>
+          <t>Corbin Carroll</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>ATL @ BAL</t>
+          <t>ARI @ WSH</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -22531,143 +22531,143 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>RF</t>
         </is>
       </c>
       <c r="J26" s="3" t="n">
-        <v>10.03</v>
+        <v>9.99</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>8.32</v>
+        <v>8.43</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>8.32</v>
+        <v>8.43</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>5.89</v>
+        <v>7.23</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>8.619999999999999</v>
+        <v>6.36</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>7.74</v>
+        <v>6.23</v>
       </c>
       <c r="P26" s="3" t="n">
-        <v>7.52</v>
+        <v>7.44</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>7.7</v>
+        <v>6.23</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>1.029</v>
+        <v>0.837</v>
       </c>
       <c r="S26" s="3" t="n">
-        <v>15.6</v>
+        <v>10.6</v>
       </c>
       <c r="T26" s="3" t="n">
-        <v>13.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="U26" s="3" t="n">
-        <v>12.4</v>
+        <v>7.53</v>
       </c>
       <c r="V26" s="4" t="inlineStr">
         <is>
-          <t>14|14|6|0|44</t>
+          <t>12|24|10|5|2</t>
         </is>
       </c>
       <c r="W26" s="4" t="inlineStr">
         <is>
-          <t>14|14|6|0|44|8|32|9|5|0</t>
+          <t>12|24|10|5|2|16|0|2|11|5</t>
         </is>
       </c>
       <c r="X26" s="4" t="inlineStr">
         <is>
-          <t>14|14|6|0|44|8|32|9|5|0|12|5|2|8|27</t>
+          <t>12|24|10|5|2|16|0|2|11|5|4|2|7|9|4</t>
         </is>
       </c>
       <c r="Y26" s="5" t="n">
-        <v>86.2</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="Z26" s="5" t="n">
-        <v>76.40000000000001</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="AA26" s="5" t="n">
-        <v>75.90000000000001</v>
+        <v>85.3</v>
       </c>
       <c r="AB26" s="5" t="n">
-        <v>70.3</v>
+        <v>75.8</v>
       </c>
       <c r="AC26" s="5" t="n">
-        <v>69.3</v>
+        <v>74.8</v>
       </c>
       <c r="AD26" s="5" t="n">
-        <v>58.6</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="AE26" s="5" t="n">
-        <v>58.1</v>
-      </c>
-      <c r="AF26" s="6" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="AG26" s="7" t="n">
-        <v>52.4</v>
+        <v>69.59999999999999</v>
+      </c>
+      <c r="AF26" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="AG26" s="6" t="n">
+        <v>55.3</v>
       </c>
       <c r="AH26" s="7" t="n">
-        <v>44.8</v>
+        <v>54.8</v>
       </c>
       <c r="AI26" s="7" t="n">
-        <v>44.3</v>
-      </c>
-      <c r="AJ26" s="8" t="n">
-        <v>37.8</v>
-      </c>
-      <c r="AK26" s="8" t="n">
-        <v>36.8</v>
+        <v>47.4</v>
+      </c>
+      <c r="AJ26" s="7" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="AK26" s="7" t="n">
+        <v>40.3</v>
       </c>
       <c r="AL26" s="8" t="n">
-        <v>32.9</v>
+        <v>35.8</v>
       </c>
       <c r="AM26" s="8" t="n">
-        <v>32.9</v>
+        <v>35.8</v>
       </c>
       <c r="AN26" s="8" t="n">
-        <v>32.9</v>
+        <v>30.9</v>
       </c>
       <c r="AO26" s="8" t="n">
-        <v>29</v>
+        <v>30.9</v>
       </c>
       <c r="AP26" s="8" t="n">
-        <v>29</v>
+        <v>28.3</v>
       </c>
       <c r="AQ26" s="8" t="n">
-        <v>26.9</v>
+        <v>24.7</v>
       </c>
       <c r="AR26" s="8" t="n">
-        <v>26.9</v>
+        <v>24.7</v>
       </c>
       <c r="AS26" s="8" t="n">
-        <v>24.4</v>
+        <v>22.7</v>
       </c>
       <c r="AT26" s="8" t="n">
-        <v>24.4</v>
+        <v>22.7</v>
       </c>
       <c r="AU26" s="8" t="n">
-        <v>22.6</v>
+        <v>18.8</v>
       </c>
       <c r="AV26" s="8" t="n">
-        <v>22.6</v>
+        <v>17.2</v>
       </c>
       <c r="AW26" s="8" t="n">
-        <v>18.7</v>
+        <v>17.2</v>
       </c>
       <c r="AX26" s="8" t="n">
-        <v>18.7</v>
+        <v>14.5</v>
       </c>
       <c r="AY26" s="8" t="n">
-        <v>17.8</v>
+        <v>14.5</v>
       </c>
       <c r="AZ26" s="3" t="n">
-        <v>219.81</v>
+        <v>219.64</v>
       </c>
       <c r="BA26" s="4" t="inlineStr">
         <is>
@@ -22676,7 +22676,7 @@
       </c>
       <c r="BB26" s="9" t="inlineStr">
         <is>
-          <t>MORE 5.5 | 58.1% | Edge +2.8</t>
+          <t>MORE 6.0 | 59.0% | Edge +2.4</t>
         </is>
       </c>
       <c r="BC26" s="4" t="inlineStr">
@@ -22685,16 +22685,16 @@
         </is>
       </c>
       <c r="BD26" s="3" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="BE26" s="3" t="n">
-        <v>58.1</v>
+        <v>59</v>
       </c>
       <c r="BF26" s="3" t="n">
-        <v>2.82</v>
+        <v>2.43</v>
       </c>
       <c r="BG26" s="3" t="n">
-        <v>16.2</v>
+        <v>18</v>
       </c>
       <c r="BH26" s="4" t="inlineStr">
         <is>
@@ -22702,7 +22702,7 @@
         </is>
       </c>
       <c r="BI26" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BJ26" s="4" t="inlineStr">
         <is>
@@ -22711,24 +22711,24 @@
       </c>
       <c r="BK26" s="4" t="n"/>
       <c r="BL26" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BM26" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="BN26" s="4" t="inlineStr">
         <is>
-          <t>1-1-1-1-1-1-1</t>
+          <t>1-3-3-3-3-3</t>
         </is>
       </c>
       <c r="BO26" s="3" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="BP26" s="3" t="n">
         <v>97</v>
       </c>
       <c r="BQ26" s="3" t="n">
-        <v>5.13</v>
+        <v>4.92</v>
       </c>
       <c r="BR26" s="4" t="inlineStr">
         <is>
@@ -22743,60 +22743,60 @@
       </c>
       <c r="BU26" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Carson Palmquist</t>
         </is>
       </c>
       <c r="BV26" s="4" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="BW26" s="3" t="n">
-        <v>4.2</v>
+        <v>8.74</v>
       </c>
       <c r="BX26" s="3" t="n">
-        <v>1.25</v>
+        <v>1.68</v>
       </c>
       <c r="BY26" s="3" t="n">
-        <v>0.224</v>
+        <v>0.2963</v>
       </c>
       <c r="BZ26" s="3" t="n">
-        <v>0.03</v>
+        <v>0.0185</v>
       </c>
       <c r="CA26" s="3" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.0556</v>
       </c>
       <c r="CB26" s="3" t="n">
-        <v>4.2</v>
+        <v>4.79</v>
       </c>
       <c r="CC26" s="3" t="n">
-        <v>1.34</v>
+        <v>1.4</v>
       </c>
       <c r="CD26" s="3" t="n">
-        <v>0.2241</v>
+        <v>0.2302</v>
       </c>
       <c r="CE26" s="3" t="n">
-        <v>0.0283</v>
+        <v>0.0356</v>
       </c>
       <c r="CF26" s="4" t="inlineStr">
         <is>
-          <t>Oriole Park at Camden Yards</t>
+          <t>Nationals Park</t>
         </is>
       </c>
       <c r="CG26" s="3" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="CH26" s="3" t="n">
         <v>1.03</v>
       </c>
       <c r="CI26" s="3" t="n">
-        <v>80.7</v>
+        <v>81.8</v>
       </c>
       <c r="CJ26" s="3" t="n">
-        <v>6.7</v>
+        <v>7.7</v>
       </c>
       <c r="CK26" s="3" t="n">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="CL26" s="3" t="n">
         <v>0</v>
@@ -22807,69 +22807,69 @@
         </is>
       </c>
       <c r="CN26" s="3" t="n">
-        <v>352</v>
+        <v>425</v>
       </c>
       <c r="CO26" s="3" t="n">
-        <v>306</v>
+        <v>370</v>
       </c>
       <c r="CP26" s="3" t="n">
-        <v>0.275</v>
+        <v>0.251</v>
       </c>
       <c r="CQ26" s="3" t="n">
-        <v>0.366</v>
+        <v>0.341</v>
       </c>
       <c r="CR26" s="3" t="n">
-        <v>0.48</v>
+        <v>0.492</v>
       </c>
       <c r="CS26" s="3" t="n">
-        <v>0.846</v>
+        <v>0.833</v>
       </c>
       <c r="CT26" s="3" t="n">
-        <v>211</v>
+        <v>130</v>
       </c>
       <c r="CU26" s="3" t="n">
-        <v>0.892</v>
+        <v>1.015</v>
       </c>
       <c r="CV26" s="3" t="n">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="CW26" s="3" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="CX26" s="3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="CY26" s="3" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="CZ26" s="3" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="DA26" s="3" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="DB26" s="3" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="DC26" s="3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="DD26" s="3" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="DE26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 vs San Diego Padres: 14 FS|2026-07-22 vs San Diego Padres: 14 FS|2026-07-21 vs San Diego Padres: 6 FS|2026-07-20 vs San Diego Padres: 0 FS|2026-07-19 vs Texas Rangers: 44 FS</t>
+          <t>2026-07-23 @ St. Louis Cardinals: 12 FS|2026-07-22 vs Athletics: 24 FS|2026-07-21 vs Athletics: 10 FS|2026-07-19 vs St. Louis Cardinals: 5 FS|2026-07-18 vs St. Louis Cardinals: 2 FS</t>
         </is>
       </c>
       <c r="DF26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 vs San Diego Padres: 14 FS|2026-07-22 vs San Diego Padres: 14 FS|2026-07-21 vs San Diego Padres: 6 FS|2026-07-20 vs San Diego Padres: 0 FS|2026-07-19 vs Texas Rangers: 44 FS|2026-07-18 vs Texas Rangers: 8 FS|2026-07-17 vs Texas Rangers: 32 FS|2026-07-12 @ St. Louis Cardinals: 9 FS|2026-07-11 @ St. Louis Cardinals: 5 FS|2026-07-10 @ St. Louis Cardinals: 0 FS</t>
+          <t>2026-07-23 @ St. Louis Cardinals: 12 FS|2026-07-22 vs Athletics: 24 FS|2026-07-21 vs Athletics: 10 FS|2026-07-19 vs St. Louis Cardinals: 5 FS|2026-07-18 vs St. Louis Cardinals: 2 FS|2026-07-17 vs St. Louis Cardinals: 16 FS|2026-07-12 @ Los Angeles Dodgers: 0 FS|2026-07-11 @ Los Angeles Dodgers: 2 FS|2026-07-10 @ Los Angeles Dodgers: 11 FS|2026-07-09 @ San Diego Padres: 5 FS</t>
         </is>
       </c>
       <c r="DG26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 vs San Diego Padres: 14 FS|2026-07-22 vs San Diego Padres: 14 FS|2026-07-21 vs San Diego Padres: 6 FS|2026-07-20 vs San Diego Padres: 0 FS|2026-07-19 vs Texas Rangers: 44 FS|2026-07-18 vs Texas Rangers: 8 FS|2026-07-17 vs Texas Rangers: 32 FS|2026-07-12 @ St. Louis Cardinals: 9 FS|2026-07-11 @ St. Louis Cardinals: 5 FS|2026-07-10 @ St. Louis Cardinals: 0 FS|2026-07-09 @ Pittsburgh Pirates: 12 FS|2026-07-08 @ Pittsburgh Pirates: 5 FS|2026-07-07 @ Pittsburgh Pirates: 2 FS|2026-07-06 vs New York Mets: 8 FS|2026-07-05 vs New York Mets: 27 FS</t>
+          <t>2026-07-23 @ St. Louis Cardinals: 12 FS|2026-07-22 vs Athletics: 24 FS|2026-07-21 vs Athletics: 10 FS|2026-07-19 vs St. Louis Cardinals: 5 FS|2026-07-18 vs St. Louis Cardinals: 2 FS|2026-07-17 vs St. Louis Cardinals: 16 FS|2026-07-12 @ Los Angeles Dodgers: 0 FS|2026-07-11 @ Los Angeles Dodgers: 2 FS|2026-07-10 @ Los Angeles Dodgers: 11 FS|2026-07-09 @ San Diego Padres: 5 FS|2026-07-08 @ San Diego Padres: 4 FS|2026-07-07 @ San Diego Padres: 2 FS|2026-07-06 @ San Diego Padres: 7 FS|2026-07-05 vs Milwaukee Brewers: 9 FS|2026-07-04 vs Milwaukee Brewers: 4 FS</t>
         </is>
       </c>
       <c r="DH26" s="3" t="n">
@@ -22879,10 +22879,10 @@
         <v>30</v>
       </c>
       <c r="DJ26" s="3" t="n">
-        <v>7.33</v>
+        <v>7.17</v>
       </c>
       <c r="DK26" s="3" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="DL26" s="4" t="inlineStr">
         <is>
@@ -22890,54 +22890,54 @@
         </is>
       </c>
       <c r="DM26" s="3" t="n">
-        <v>16.86</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="DN26" s="3" t="n">
-        <v>11.36</v>
+        <v>7.79</v>
       </c>
       <c r="DO26" s="3" t="n">
-        <v>0.392</v>
+        <v>0.167</v>
       </c>
       <c r="DP26" s="4" t="inlineStr">
         <is>
-          <t>Hot</t>
+          <t>Cold</t>
         </is>
       </c>
       <c r="DQ26" s="3" t="n">
-        <v>7.33</v>
+        <v>7.17</v>
       </c>
       <c r="DR26" s="3" t="n">
-        <v>2.524</v>
+        <v>1.758</v>
       </c>
       <c r="DS26" s="3" t="n">
-        <v>0.3175</v>
+        <v>0.1452</v>
       </c>
       <c r="DT26" s="3" t="n">
-        <v>0.0635</v>
+        <v>0.1129</v>
       </c>
       <c r="DU26" s="3" t="n">
-        <v>0.0635</v>
+        <v>0.0323</v>
       </c>
       <c r="DV26" s="3" t="n">
-        <v>0.1746</v>
+        <v>0.1129</v>
       </c>
       <c r="DW26" s="3" t="n">
-        <v>0.0159</v>
+        <v>0.0323</v>
       </c>
       <c r="DX26" s="3" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="DY26" s="3" t="n">
+        <v>9.34</v>
+      </c>
+      <c r="DZ26" s="3" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="EA26" s="3" t="n">
         <v>10.12</v>
       </c>
-      <c r="DY26" s="3" t="n">
-        <v>8.93</v>
-      </c>
-      <c r="DZ26" s="3" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="EA26" s="3" t="n">
-        <v>11.34</v>
-      </c>
       <c r="EB26" s="3" t="n">
-        <v>9.19</v>
+        <v>9.99</v>
       </c>
       <c r="EC26" s="3" t="n">
         <v>28</v>
@@ -22955,25 +22955,25 @@
         <v>20</v>
       </c>
       <c r="EH26" s="3" t="n">
-        <v>170</v>
+        <v>265</v>
       </c>
       <c r="EI26" s="3" t="n">
-        <v>84.79000000000001</v>
+        <v>84.8</v>
       </c>
       <c r="EJ26" s="3" t="n">
-        <v>28.24</v>
+        <v>28.3</v>
       </c>
       <c r="EK26" s="3" t="n">
-        <v>2.94</v>
+        <v>0.75</v>
       </c>
       <c r="EL26" s="3" t="n">
-        <v>28.24</v>
+        <v>24.53</v>
       </c>
       <c r="EM26" s="3" t="n">
-        <v>0.385</v>
+        <v>0.365</v>
       </c>
       <c r="EN26" s="3" t="n">
-        <v>0.958</v>
+        <v>0.926</v>
       </c>
       <c r="EO26" s="3" t="n">
         <v>1</v>
@@ -22985,74 +22985,74 @@
         <v>1</v>
       </c>
       <c r="ER26" s="3" t="n">
-        <v>1</v>
+        <v>0.9426</v>
       </c>
       <c r="ES26" s="3" t="n">
-        <v>0</v>
+        <v>547</v>
       </c>
       <c r="ET26" s="4" t="inlineStr">
         <is>
+          <t>Statcast</t>
+        </is>
+      </c>
+      <c r="EU26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="EV26" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="EW26" s="4" t="inlineStr">
+        <is>
           <t>Fallback</t>
         </is>
       </c>
-      <c r="EU26" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="EV26" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="EW26" s="4" t="inlineStr">
-        <is>
-          <t>Fallback</t>
-        </is>
-      </c>
       <c r="EX26" s="3" t="n">
-        <v>170</v>
+        <v>265</v>
       </c>
       <c r="EY26" s="3" t="n">
-        <v>84.79000000000001</v>
+        <v>84.8</v>
       </c>
       <c r="EZ26" s="3" t="n">
         <v>12</v>
       </c>
       <c r="FA26" s="3" t="n">
-        <v>16.58</v>
+        <v>20.71</v>
       </c>
       <c r="FB26" s="3" t="n">
-        <v>30.41</v>
+        <v>35</v>
       </c>
       <c r="FC26" s="3" t="n">
-        <v>17.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="FD26" s="3" t="n">
-        <v>65.90000000000001</v>
+        <v>62.3</v>
       </c>
       <c r="FE26" s="3" t="n">
-        <v>16.5</v>
+        <v>27.9</v>
       </c>
       <c r="FF26" s="3" t="n">
-        <v>1.0181</v>
+        <v>1.0154</v>
       </c>
       <c r="FG26" s="3" t="n">
-        <v>1.0032</v>
+        <v>1.0049</v>
       </c>
       <c r="FH26" s="3" t="n">
-        <v>1.0299</v>
+        <v>1.0338</v>
       </c>
       <c r="FI26" s="3" t="n">
-        <v>1.0063</v>
+        <v>1.0099</v>
       </c>
       <c r="FJ26" s="3" t="n">
-        <v>1.0396</v>
+        <v>1.0489</v>
       </c>
       <c r="FK26" s="3" t="n">
-        <v>1.0498</v>
+        <v>1.0163</v>
       </c>
       <c r="FL26" s="3" t="n">
-        <v>11.49</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="FM26" s="3" t="n">
-        <v>4.15</v>
+        <v>1.36</v>
       </c>
       <c r="FN26" s="4" t="inlineStr">
         <is>
@@ -23097,7 +23097,7 @@
         <v>27</v>
       </c>
       <c r="FZ26" s="3" t="n">
-        <v>0.9139</v>
+        <v>1.3</v>
       </c>
       <c r="GA26" s="3" t="n">
         <v>27</v>
@@ -23106,43 +23106,43 @@
         <v>1</v>
       </c>
       <c r="GC26" s="3" t="n">
-        <v>0.1658</v>
+        <v>0.1613</v>
       </c>
       <c r="GD26" s="3" t="n">
-        <v>0.031</v>
+        <v>0.0606</v>
       </c>
       <c r="GE26" s="3" t="n">
-        <v>0.0028</v>
+        <v>0.0116</v>
       </c>
       <c r="GF26" s="3" t="n">
-        <v>0.0451</v>
+        <v>0.0288</v>
       </c>
       <c r="GG26" s="3" t="n">
-        <v>0.108</v>
+        <v>0.0774</v>
       </c>
       <c r="GH26" s="3" t="n">
-        <v>0.0143</v>
+        <v>0.0075</v>
       </c>
       <c r="GI26" s="3" t="n">
-        <v>0.2104</v>
+        <v>0.2335</v>
       </c>
       <c r="GJ26" s="3" t="n">
-        <v>0.4811</v>
+        <v>0.5194</v>
       </c>
       <c r="GK26" s="3" t="n">
-        <v>0.2531</v>
+        <v>0.31</v>
       </c>
       <c r="GL26" s="3" t="n">
-        <v>0.2658</v>
+        <v>0.1705</v>
       </c>
       <c r="GM26" s="3" t="n">
-        <v>0.1423</v>
+        <v>0.1495</v>
       </c>
       <c r="GN26" s="3" t="n">
-        <v>0.1253</v>
+        <v>0.1452</v>
       </c>
       <c r="GO26" s="3" t="n">
-        <v>0.0102</v>
+        <v>0.0207</v>
       </c>
       <c r="GP26" s="3" t="n">
         <v>1</v>
@@ -23154,19 +23154,19 @@
       </c>
       <c r="GR26" s="4" t="n"/>
       <c r="GS26" s="3" t="n">
-        <v>7.7</v>
+        <v>6.23</v>
       </c>
       <c r="GT26" s="3" t="n">
-        <v>2.8</v>
+        <v>3.88</v>
       </c>
       <c r="GU26" s="3" t="n">
-        <v>12.07</v>
+        <v>11.42</v>
       </c>
       <c r="GV26" s="3" t="n">
-        <v>19.27</v>
+        <v>17.28</v>
       </c>
       <c r="GW26" s="3" t="n">
-        <v>4.5</v>
+        <v>4.49</v>
       </c>
       <c r="GX26" s="3" t="n">
         <v>0</v>
@@ -23182,91 +23182,91 @@
         </is>
       </c>
       <c r="HA26" s="3" t="n">
-        <v>78.2</v>
+        <v>84.3</v>
       </c>
       <c r="HB26" s="3" t="n">
-        <v>68.40000000000001</v>
+        <v>84.3</v>
       </c>
       <c r="HC26" s="3" t="n">
-        <v>68.40000000000001</v>
+        <v>77.8</v>
       </c>
       <c r="HD26" s="3" t="n">
-        <v>63.3</v>
+        <v>68.8</v>
       </c>
       <c r="HE26" s="3" t="n">
-        <v>63.3</v>
+        <v>68.8</v>
       </c>
       <c r="HF26" s="3" t="n">
-        <v>53.6</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="HG26" s="3" t="n">
-        <v>53.6</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="HH26" s="3" t="n">
-        <v>48.9</v>
+        <v>55</v>
       </c>
       <c r="HI26" s="3" t="n">
-        <v>48.9</v>
+        <v>51.8</v>
       </c>
       <c r="HJ26" s="3" t="n">
-        <v>41.8</v>
+        <v>51.8</v>
       </c>
       <c r="HK26" s="3" t="n">
-        <v>41.8</v>
+        <v>44.9</v>
       </c>
       <c r="HL26" s="3" t="n">
-        <v>36.8</v>
+        <v>44.9</v>
       </c>
       <c r="HM26" s="3" t="n">
-        <v>36.8</v>
+        <v>40.3</v>
       </c>
       <c r="HN26" s="3" t="n">
-        <v>32.9</v>
+        <v>35.8</v>
       </c>
       <c r="HO26" s="3" t="n">
-        <v>32.9</v>
+        <v>35.8</v>
       </c>
       <c r="HP26" s="3" t="n">
-        <v>32.9</v>
+        <v>30.9</v>
       </c>
       <c r="HQ26" s="3" t="n">
-        <v>29</v>
+        <v>30.9</v>
       </c>
       <c r="HR26" s="3" t="n">
-        <v>29</v>
+        <v>28.3</v>
       </c>
       <c r="HS26" s="3" t="n">
-        <v>26.9</v>
+        <v>24.7</v>
       </c>
       <c r="HT26" s="3" t="n">
-        <v>26.9</v>
+        <v>24.7</v>
       </c>
       <c r="HU26" s="3" t="n">
-        <v>24.4</v>
+        <v>22.7</v>
       </c>
       <c r="HV26" s="3" t="n">
-        <v>24.4</v>
+        <v>22.7</v>
       </c>
       <c r="HW26" s="3" t="n">
-        <v>22.6</v>
+        <v>18.8</v>
       </c>
       <c r="HX26" s="3" t="n">
-        <v>22.6</v>
+        <v>17.2</v>
       </c>
       <c r="HY26" s="3" t="n">
-        <v>18.7</v>
+        <v>17.2</v>
       </c>
       <c r="HZ26" s="3" t="n">
-        <v>18.7</v>
+        <v>14.5</v>
       </c>
       <c r="IA26" s="3" t="n">
-        <v>17.8</v>
+        <v>14.5</v>
       </c>
       <c r="IB26" s="3" t="n">
-        <v>8</v>
+        <v>6.3</v>
       </c>
       <c r="IC26" s="3" t="n">
-        <v>8</v>
+        <v>6.3</v>
       </c>
       <c r="ID26" s="3" t="n">
         <v>7.5</v>
@@ -23358,22 +23358,22 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Corbin Carroll</t>
+          <t>Drake Baldwin</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>ARI @ WSH</t>
+          <t>ATL @ BAL</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -23383,140 +23383,140 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J27" s="3" t="n">
-        <v>9.99</v>
+        <v>10.03</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>8.43</v>
+        <v>8.31</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>8.43</v>
+        <v>8.31</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>7.23</v>
+        <v>5.89</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>6.36</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>6.23</v>
+        <v>7.74</v>
       </c>
       <c r="P27" s="3" t="n">
-        <v>7.44</v>
+        <v>7.52</v>
       </c>
       <c r="Q27" s="3" t="n">
-        <v>6.23</v>
+        <v>7.7</v>
       </c>
       <c r="R27" s="3" t="n">
-        <v>0.837</v>
+        <v>1.029</v>
       </c>
       <c r="S27" s="3" t="n">
-        <v>10.6</v>
+        <v>15.6</v>
       </c>
       <c r="T27" s="3" t="n">
-        <v>8.699999999999999</v>
+        <v>13.2</v>
       </c>
       <c r="U27" s="3" t="n">
-        <v>7.53</v>
+        <v>12.4</v>
       </c>
       <c r="V27" s="4" t="inlineStr">
         <is>
-          <t>12|24|10|5|2</t>
+          <t>14|14|6|0|44</t>
         </is>
       </c>
       <c r="W27" s="4" t="inlineStr">
         <is>
-          <t>12|24|10|5|2|16|0|2|11|5</t>
+          <t>14|14|6|0|44|8|32|9|5|0</t>
         </is>
       </c>
       <c r="X27" s="4" t="inlineStr">
         <is>
-          <t>12|24|10|5|2|16|0|2|11|5|4|2|7|9|4</t>
+          <t>14|14|6|0|44|8|32|9|5|0|12|5|2|8|27</t>
         </is>
       </c>
       <c r="Y27" s="5" t="n">
-        <v>90.59999999999999</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="Z27" s="5" t="n">
-        <v>90.59999999999999</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="AA27" s="5" t="n">
-        <v>85.3</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="AB27" s="5" t="n">
-        <v>75.8</v>
+        <v>70.3</v>
       </c>
       <c r="AC27" s="5" t="n">
-        <v>74.8</v>
+        <v>69.3</v>
       </c>
       <c r="AD27" s="5" t="n">
-        <v>70.09999999999999</v>
+        <v>58.5</v>
       </c>
       <c r="AE27" s="5" t="n">
-        <v>69.59999999999999</v>
-      </c>
-      <c r="AF27" s="5" t="n">
-        <v>59</v>
-      </c>
-      <c r="AG27" s="6" t="n">
-        <v>55.3</v>
+        <v>58</v>
+      </c>
+      <c r="AF27" s="6" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="AG27" s="7" t="n">
+        <v>52.3</v>
       </c>
       <c r="AH27" s="7" t="n">
-        <v>54.8</v>
+        <v>44.7</v>
       </c>
       <c r="AI27" s="7" t="n">
-        <v>47.4</v>
-      </c>
-      <c r="AJ27" s="7" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="AK27" s="7" t="n">
-        <v>40.3</v>
+        <v>44.2</v>
+      </c>
+      <c r="AJ27" s="8" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="AK27" s="8" t="n">
+        <v>36.7</v>
       </c>
       <c r="AL27" s="8" t="n">
-        <v>35.8</v>
+        <v>32.8</v>
       </c>
       <c r="AM27" s="8" t="n">
-        <v>35.8</v>
+        <v>32.8</v>
       </c>
       <c r="AN27" s="8" t="n">
-        <v>30.9</v>
+        <v>32.8</v>
       </c>
       <c r="AO27" s="8" t="n">
-        <v>30.9</v>
+        <v>28.9</v>
       </c>
       <c r="AP27" s="8" t="n">
-        <v>28.3</v>
+        <v>28.9</v>
       </c>
       <c r="AQ27" s="8" t="n">
-        <v>24.7</v>
+        <v>26.9</v>
       </c>
       <c r="AR27" s="8" t="n">
-        <v>24.7</v>
+        <v>26.9</v>
       </c>
       <c r="AS27" s="8" t="n">
-        <v>22.7</v>
+        <v>24.4</v>
       </c>
       <c r="AT27" s="8" t="n">
-        <v>22.7</v>
+        <v>24.4</v>
       </c>
       <c r="AU27" s="8" t="n">
-        <v>18.8</v>
+        <v>22.6</v>
       </c>
       <c r="AV27" s="8" t="n">
-        <v>17.2</v>
+        <v>22.6</v>
       </c>
       <c r="AW27" s="8" t="n">
-        <v>17.2</v>
+        <v>18.7</v>
       </c>
       <c r="AX27" s="8" t="n">
-        <v>14.5</v>
+        <v>18.7</v>
       </c>
       <c r="AY27" s="8" t="n">
-        <v>14.5</v>
+        <v>17.8</v>
       </c>
       <c r="AZ27" s="3" t="n">
         <v>219.64</v>
@@ -23528,7 +23528,7 @@
       </c>
       <c r="BB27" s="9" t="inlineStr">
         <is>
-          <t>MORE 6.0 | 59.0% | Edge +2.4</t>
+          <t>MORE 5.5 | 58.0% | Edge +2.8</t>
         </is>
       </c>
       <c r="BC27" s="4" t="inlineStr">
@@ -23537,16 +23537,16 @@
         </is>
       </c>
       <c r="BD27" s="3" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="BE27" s="3" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="BF27" s="3" t="n">
-        <v>2.43</v>
+        <v>2.81</v>
       </c>
       <c r="BG27" s="3" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="BH27" s="4" t="inlineStr">
         <is>
@@ -23554,7 +23554,7 @@
         </is>
       </c>
       <c r="BI27" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BJ27" s="4" t="inlineStr">
         <is>
@@ -23563,24 +23563,24 @@
       </c>
       <c r="BK27" s="4" t="n"/>
       <c r="BL27" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BM27" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="BN27" s="4" t="inlineStr">
         <is>
-          <t>1-3-3-3-3-3</t>
+          <t>1-1-1-1-1-1-1</t>
         </is>
       </c>
       <c r="BO27" s="3" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="BP27" s="3" t="n">
         <v>97</v>
       </c>
       <c r="BQ27" s="3" t="n">
-        <v>4.92</v>
+        <v>5.13</v>
       </c>
       <c r="BR27" s="4" t="inlineStr">
         <is>
@@ -23595,60 +23595,60 @@
       </c>
       <c r="BU27" s="4" t="inlineStr">
         <is>
-          <t>Carson Palmquist</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="BV27" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="BW27" s="3" t="n">
-        <v>8.74</v>
+        <v>4.2</v>
       </c>
       <c r="BX27" s="3" t="n">
-        <v>1.68</v>
+        <v>1.25</v>
       </c>
       <c r="BY27" s="3" t="n">
-        <v>0.2963</v>
+        <v>0.224</v>
       </c>
       <c r="BZ27" s="3" t="n">
-        <v>0.0185</v>
+        <v>0.03</v>
       </c>
       <c r="CA27" s="3" t="n">
-        <v>0.0556</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="CB27" s="3" t="n">
-        <v>4.79</v>
+        <v>4.2</v>
       </c>
       <c r="CC27" s="3" t="n">
-        <v>1.4</v>
+        <v>1.34</v>
       </c>
       <c r="CD27" s="3" t="n">
-        <v>0.2302</v>
+        <v>0.2241</v>
       </c>
       <c r="CE27" s="3" t="n">
-        <v>0.0356</v>
+        <v>0.0283</v>
       </c>
       <c r="CF27" s="4" t="inlineStr">
         <is>
-          <t>Nationals Park</t>
+          <t>Oriole Park at Camden Yards</t>
         </is>
       </c>
       <c r="CG27" s="3" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="CH27" s="3" t="n">
         <v>1.03</v>
       </c>
       <c r="CI27" s="3" t="n">
-        <v>81.8</v>
+        <v>80.7</v>
       </c>
       <c r="CJ27" s="3" t="n">
-        <v>7.7</v>
+        <v>6.7</v>
       </c>
       <c r="CK27" s="3" t="n">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="CL27" s="3" t="n">
         <v>0</v>
@@ -23659,69 +23659,69 @@
         </is>
       </c>
       <c r="CN27" s="3" t="n">
-        <v>425</v>
+        <v>352</v>
       </c>
       <c r="CO27" s="3" t="n">
-        <v>370</v>
+        <v>306</v>
       </c>
       <c r="CP27" s="3" t="n">
-        <v>0.251</v>
+        <v>0.275</v>
       </c>
       <c r="CQ27" s="3" t="n">
-        <v>0.341</v>
+        <v>0.366</v>
       </c>
       <c r="CR27" s="3" t="n">
-        <v>0.492</v>
+        <v>0.48</v>
       </c>
       <c r="CS27" s="3" t="n">
-        <v>0.833</v>
+        <v>0.846</v>
       </c>
       <c r="CT27" s="3" t="n">
-        <v>130</v>
+        <v>211</v>
       </c>
       <c r="CU27" s="3" t="n">
-        <v>1.015</v>
+        <v>0.892</v>
       </c>
       <c r="CV27" s="3" t="n">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="CW27" s="3" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="CX27" s="3" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="CY27" s="3" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="CZ27" s="3" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="DA27" s="3" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="DB27" s="3" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="DC27" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="DD27" s="3" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="DE27" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 @ St. Louis Cardinals: 12 FS|2026-07-22 vs Athletics: 24 FS|2026-07-21 vs Athletics: 10 FS|2026-07-19 vs St. Louis Cardinals: 5 FS|2026-07-18 vs St. Louis Cardinals: 2 FS</t>
+          <t>2026-07-23 vs San Diego Padres: 14 FS|2026-07-22 vs San Diego Padres: 14 FS|2026-07-21 vs San Diego Padres: 6 FS|2026-07-20 vs San Diego Padres: 0 FS|2026-07-19 vs Texas Rangers: 44 FS</t>
         </is>
       </c>
       <c r="DF27" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 @ St. Louis Cardinals: 12 FS|2026-07-22 vs Athletics: 24 FS|2026-07-21 vs Athletics: 10 FS|2026-07-19 vs St. Louis Cardinals: 5 FS|2026-07-18 vs St. Louis Cardinals: 2 FS|2026-07-17 vs St. Louis Cardinals: 16 FS|2026-07-12 @ Los Angeles Dodgers: 0 FS|2026-07-11 @ Los Angeles Dodgers: 2 FS|2026-07-10 @ Los Angeles Dodgers: 11 FS|2026-07-09 @ San Diego Padres: 5 FS</t>
+          <t>2026-07-23 vs San Diego Padres: 14 FS|2026-07-22 vs San Diego Padres: 14 FS|2026-07-21 vs San Diego Padres: 6 FS|2026-07-20 vs San Diego Padres: 0 FS|2026-07-19 vs Texas Rangers: 44 FS|2026-07-18 vs Texas Rangers: 8 FS|2026-07-17 vs Texas Rangers: 32 FS|2026-07-12 @ St. Louis Cardinals: 9 FS|2026-07-11 @ St. Louis Cardinals: 5 FS|2026-07-10 @ St. Louis Cardinals: 0 FS</t>
         </is>
       </c>
       <c r="DG27" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23 @ St. Louis Cardinals: 12 FS|2026-07-22 vs Athletics: 24 FS|2026-07-21 vs Athletics: 10 FS|2026-07-19 vs St. Louis Cardinals: 5 FS|2026-07-18 vs St. Louis Cardinals: 2 FS|2026-07-17 vs St. Louis Cardinals: 16 FS|2026-07-12 @ Los Angeles Dodgers: 0 FS|2026-07-11 @ Los Angeles Dodgers: 2 FS|2026-07-10 @ Los Angeles Dodgers: 11 FS|2026-07-09 @ San Diego Padres: 5 FS|2026-07-08 @ San Diego Padres: 4 FS|2026-07-07 @ San Diego Padres: 2 FS|2026-07-06 @ San Diego Padres: 7 FS|2026-07-05 vs Milwaukee Brewers: 9 FS|2026-07-04 vs Milwaukee Brewers: 4 FS</t>
+          <t>2026-07-23 vs San Diego Padres: 14 FS|2026-07-22 vs San Diego Padres: 14 FS|2026-07-21 vs San Diego Padres: 6 FS|2026-07-20 vs San Diego Padres: 0 FS|2026-07-19 vs Texas Rangers: 44 FS|2026-07-18 vs Texas Rangers: 8 FS|2026-07-17 vs Texas Rangers: 32 FS|2026-07-12 @ St. Louis Cardinals: 9 FS|2026-07-11 @ St. Louis Cardinals: 5 FS|2026-07-10 @ St. Louis Cardinals: 0 FS|2026-07-09 @ Pittsburgh Pirates: 12 FS|2026-07-08 @ Pittsburgh Pirates: 5 FS|2026-07-07 @ Pittsburgh Pirates: 2 FS|2026-07-06 vs New York Mets: 8 FS|2026-07-05 vs New York Mets: 27 FS</t>
         </is>
       </c>
       <c r="DH27" s="3" t="n">
@@ -23731,10 +23731,10 @@
         <v>30</v>
       </c>
       <c r="DJ27" s="3" t="n">
-        <v>7.17</v>
+        <v>7.33</v>
       </c>
       <c r="DK27" s="3" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="DL27" s="4" t="inlineStr">
         <is>
@@ -23742,54 +23742,54 @@
         </is>
       </c>
       <c r="DM27" s="3" t="n">
-        <v>9.859999999999999</v>
+        <v>16.86</v>
       </c>
       <c r="DN27" s="3" t="n">
-        <v>7.79</v>
+        <v>11.36</v>
       </c>
       <c r="DO27" s="3" t="n">
-        <v>0.167</v>
+        <v>0.392</v>
       </c>
       <c r="DP27" s="4" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Hot</t>
         </is>
       </c>
       <c r="DQ27" s="3" t="n">
-        <v>7.17</v>
+        <v>7.33</v>
       </c>
       <c r="DR27" s="3" t="n">
-        <v>1.758</v>
+        <v>2.524</v>
       </c>
       <c r="DS27" s="3" t="n">
-        <v>0.1452</v>
+        <v>0.3175</v>
       </c>
       <c r="DT27" s="3" t="n">
-        <v>0.1129</v>
+        <v>0.0635</v>
       </c>
       <c r="DU27" s="3" t="n">
-        <v>0.0323</v>
+        <v>0.0635</v>
       </c>
       <c r="DV27" s="3" t="n">
-        <v>0.1129</v>
+        <v>0.1746</v>
       </c>
       <c r="DW27" s="3" t="n">
-        <v>0.0323</v>
+        <v>0.0159</v>
       </c>
       <c r="DX27" s="3" t="n">
-        <v>10.51</v>
+        <v>10.12</v>
       </c>
       <c r="DY27" s="3" t="n">
-        <v>9.34</v>
+        <v>8.93</v>
       </c>
       <c r="DZ27" s="3" t="n">
-        <v>9.67</v>
+        <v>10.6</v>
       </c>
       <c r="EA27" s="3" t="n">
-        <v>10.12</v>
+        <v>11.34</v>
       </c>
       <c r="EB27" s="3" t="n">
-        <v>9.99</v>
+        <v>9.19</v>
       </c>
       <c r="EC27" s="3" t="n">
         <v>28</v>
@@ -23807,25 +23807,25 @@
         <v>20</v>
       </c>
       <c r="EH27" s="3" t="n">
-        <v>265</v>
+        <v>170</v>
       </c>
       <c r="EI27" s="3" t="n">
-        <v>84.8</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="EJ27" s="3" t="n">
-        <v>28.3</v>
+        <v>28.24</v>
       </c>
       <c r="EK27" s="3" t="n">
-        <v>0.75</v>
+        <v>2.94</v>
       </c>
       <c r="EL27" s="3" t="n">
-        <v>24.53</v>
+        <v>28.24</v>
       </c>
       <c r="EM27" s="3" t="n">
-        <v>0.365</v>
+        <v>0.385</v>
       </c>
       <c r="EN27" s="3" t="n">
-        <v>0.926</v>
+        <v>0.958</v>
       </c>
       <c r="EO27" s="3" t="n">
         <v>1</v>
@@ -23837,21 +23837,21 @@
         <v>1</v>
       </c>
       <c r="ER27" s="3" t="n">
-        <v>0.9426</v>
+        <v>1</v>
       </c>
       <c r="ES27" s="3" t="n">
-        <v>547</v>
+        <v>0</v>
       </c>
       <c r="ET27" s="4" t="inlineStr">
         <is>
-          <t>Statcast</t>
+          <t>Fallback</t>
         </is>
       </c>
       <c r="EU27" s="3" t="n">
         <v>1</v>
       </c>
       <c r="EV27" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="EW27" s="4" t="inlineStr">
         <is>
@@ -23859,52 +23859,52 @@
         </is>
       </c>
       <c r="EX27" s="3" t="n">
-        <v>265</v>
+        <v>170</v>
       </c>
       <c r="EY27" s="3" t="n">
-        <v>84.8</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="EZ27" s="3" t="n">
         <v>12</v>
       </c>
       <c r="FA27" s="3" t="n">
-        <v>20.71</v>
+        <v>16.58</v>
       </c>
       <c r="FB27" s="3" t="n">
-        <v>35</v>
+        <v>30.41</v>
       </c>
       <c r="FC27" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>17.6</v>
       </c>
       <c r="FD27" s="3" t="n">
-        <v>62.3</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="FE27" s="3" t="n">
-        <v>27.9</v>
+        <v>16.5</v>
       </c>
       <c r="FF27" s="3" t="n">
-        <v>1.0154</v>
+        <v>1.0181</v>
       </c>
       <c r="FG27" s="3" t="n">
-        <v>1.0049</v>
+        <v>1.0032</v>
       </c>
       <c r="FH27" s="3" t="n">
-        <v>1.0338</v>
+        <v>1.0299</v>
       </c>
       <c r="FI27" s="3" t="n">
-        <v>1.0099</v>
+        <v>1.0063</v>
       </c>
       <c r="FJ27" s="3" t="n">
-        <v>1.0489</v>
+        <v>1.0396</v>
       </c>
       <c r="FK27" s="3" t="n">
-        <v>1.0163</v>
+        <v>1.0498</v>
       </c>
       <c r="FL27" s="3" t="n">
-        <v>8.529999999999999</v>
+        <v>11.49</v>
       </c>
       <c r="FM27" s="3" t="n">
-        <v>1.36</v>
+        <v>4.15</v>
       </c>
       <c r="FN27" s="4" t="inlineStr">
         <is>
@@ -23949,7 +23949,7 @@
         <v>27</v>
       </c>
       <c r="FZ27" s="3" t="n">
-        <v>1.3</v>
+        <v>0.9139</v>
       </c>
       <c r="GA27" s="3" t="n">
         <v>27</v>
@@ -23958,43 +23958,43 @@
         <v>1</v>
       </c>
       <c r="GC27" s="3" t="n">
-        <v>0.1613</v>
+        <v>0.1658</v>
       </c>
       <c r="GD27" s="3" t="n">
-        <v>0.0606</v>
+        <v>0.031</v>
       </c>
       <c r="GE27" s="3" t="n">
-        <v>0.0116</v>
+        <v>0.0028</v>
       </c>
       <c r="GF27" s="3" t="n">
-        <v>0.0288</v>
+        <v>0.0451</v>
       </c>
       <c r="GG27" s="3" t="n">
-        <v>0.0774</v>
+        <v>0.108</v>
       </c>
       <c r="GH27" s="3" t="n">
-        <v>0.0075</v>
+        <v>0.0143</v>
       </c>
       <c r="GI27" s="3" t="n">
-        <v>0.2335</v>
+        <v>0.2104</v>
       </c>
       <c r="GJ27" s="3" t="n">
-        <v>0.5194</v>
+        <v>0.4811</v>
       </c>
       <c r="GK27" s="3" t="n">
-        <v>0.31</v>
+        <v>0.2531</v>
       </c>
       <c r="GL27" s="3" t="n">
-        <v>0.1705</v>
+        <v>0.2658</v>
       </c>
       <c r="GM27" s="3" t="n">
-        <v>0.1495</v>
+        <v>0.1423</v>
       </c>
       <c r="GN27" s="3" t="n">
-        <v>0.1452</v>
+        <v>0.1253</v>
       </c>
       <c r="GO27" s="3" t="n">
-        <v>0.0207</v>
+        <v>0.0102</v>
       </c>
       <c r="GP27" s="3" t="n">
         <v>1</v>
@@ -24006,19 +24006,19 @@
       </c>
       <c r="GR27" s="4" t="n"/>
       <c r="GS27" s="3" t="n">
-        <v>6.23</v>
+        <v>7.7</v>
       </c>
       <c r="GT27" s="3" t="n">
-        <v>3.88</v>
+        <v>2.81</v>
       </c>
       <c r="GU27" s="3" t="n">
-        <v>11.42</v>
+        <v>12.07</v>
       </c>
       <c r="GV27" s="3" t="n">
-        <v>17.28</v>
+        <v>19.27</v>
       </c>
       <c r="GW27" s="3" t="n">
-        <v>4.49</v>
+        <v>4.5</v>
       </c>
       <c r="GX27" s="3" t="n">
         <v>0</v>
@@ -24034,91 +24034,91 @@
         </is>
       </c>
       <c r="HA27" s="3" t="n">
-        <v>84.3</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="HB27" s="3" t="n">
-        <v>84.3</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="HC27" s="3" t="n">
-        <v>77.8</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="HD27" s="3" t="n">
-        <v>68.8</v>
+        <v>63.3</v>
       </c>
       <c r="HE27" s="3" t="n">
-        <v>68.8</v>
+        <v>63.3</v>
       </c>
       <c r="HF27" s="3" t="n">
-        <v>65.09999999999999</v>
+        <v>53.5</v>
       </c>
       <c r="HG27" s="3" t="n">
-        <v>65.09999999999999</v>
+        <v>53.5</v>
       </c>
       <c r="HH27" s="3" t="n">
-        <v>55</v>
+        <v>48.8</v>
       </c>
       <c r="HI27" s="3" t="n">
-        <v>51.8</v>
+        <v>48.8</v>
       </c>
       <c r="HJ27" s="3" t="n">
-        <v>51.8</v>
+        <v>41.7</v>
       </c>
       <c r="HK27" s="3" t="n">
-        <v>44.9</v>
+        <v>41.7</v>
       </c>
       <c r="HL27" s="3" t="n">
-        <v>44.9</v>
+        <v>36.7</v>
       </c>
       <c r="HM27" s="3" t="n">
-        <v>40.3</v>
+        <v>36.7</v>
       </c>
       <c r="HN27" s="3" t="n">
-        <v>35.8</v>
+        <v>32.8</v>
       </c>
       <c r="HO27" s="3" t="n">
-        <v>35.8</v>
+        <v>32.8</v>
       </c>
       <c r="HP27" s="3" t="n">
-        <v>30.9</v>
+        <v>32.8</v>
       </c>
       <c r="HQ27" s="3" t="n">
-        <v>30.9</v>
+        <v>28.9</v>
       </c>
       <c r="HR27" s="3" t="n">
-        <v>28.3</v>
+        <v>28.9</v>
       </c>
       <c r="HS27" s="3" t="n">
-        <v>24.7</v>
+        <v>26.9</v>
       </c>
       <c r="HT27" s="3" t="n">
-        <v>24.7</v>
+        <v>26.9</v>
       </c>
       <c r="HU27" s="3" t="n">
-        <v>22.7</v>
+        <v>24.4</v>
       </c>
       <c r="HV27" s="3" t="n">
-        <v>22.7</v>
+        <v>24.4</v>
       </c>
       <c r="HW27" s="3" t="n">
-        <v>18.8</v>
+        <v>22.6</v>
       </c>
       <c r="HX27" s="3" t="n">
-        <v>17.2</v>
+        <v>22.6</v>
       </c>
       <c r="HY27" s="3" t="n">
-        <v>17.2</v>
+        <v>18.7</v>
       </c>
       <c r="HZ27" s="3" t="n">
-        <v>14.5</v>
+        <v>18.7</v>
       </c>
       <c r="IA27" s="3" t="n">
-        <v>14.5</v>
+        <v>17.8</v>
       </c>
       <c r="IB27" s="3" t="n">
-        <v>6.3</v>
+        <v>8</v>
       </c>
       <c r="IC27" s="3" t="n">
-        <v>6.3</v>
+        <v>8</v>
       </c>
       <c r="ID27" s="3" t="n">
         <v>7.5</v>

</xml_diff>